<commit_message>
Capture updated LIB_FILELIST makefile and error messages
</commit_message>
<xml_diff>
--- a/var/ols_error_messages.xlsx
+++ b/var/ols_error_messages.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\olaus-J70091652\var\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\b-lib-olaus-J70091652\var\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BEACF9F-6C6E-4510-B2DE-D143831C0F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92495FAC-B480-4B03-8979-6E4142971A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32340" yWindow="2715" windowWidth="24330" windowHeight="11070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="3765" windowWidth="45030" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="73">
   <si>
     <t>Error Number</t>
   </si>
@@ -73,13 +84,184 @@
   </si>
   <si>
     <t>Argument #1 is less than or equal 0.</t>
+  </si>
+  <si>
+    <t>OLS7000I</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;</t>
+  </si>
+  <si>
+    <t>OLS7004F</t>
+  </si>
+  <si>
+    <t>OLS7006F</t>
+  </si>
+  <si>
+    <t>OLS7007F</t>
+  </si>
+  <si>
+    <t>OLS7008F</t>
+  </si>
+  <si>
+    <t>OLS7009F</t>
+  </si>
+  <si>
+    <t>OLS7010F</t>
+  </si>
+  <si>
+    <t>OLS7011F</t>
+  </si>
+  <si>
+    <t>OLS7012F</t>
+  </si>
+  <si>
+    <t>OLS7013F</t>
+  </si>
+  <si>
+    <t>OLS7014F</t>
+  </si>
+  <si>
+    <t>OLS7015F</t>
+  </si>
+  <si>
+    <t>OLS7016F</t>
+  </si>
+  <si>
+    <t>OLS7017F</t>
+  </si>
+  <si>
+    <t>OLS7018F</t>
+  </si>
+  <si>
+    <t>OLS7019F</t>
+  </si>
+  <si>
+    <t>OLS7020F</t>
+  </si>
+  <si>
+    <t>OLS7999I</t>
+  </si>
+  <si>
+    <t>ols_end</t>
+  </si>
+  <si>
+    <t>Program stops</t>
+  </si>
+  <si>
+    <t>EX_USAGE</t>
+  </si>
+  <si>
+    <t>EX_OK</t>
+  </si>
+  <si>
+    <t>assert</t>
+  </si>
+  <si>
+    <t>EX_ASSERTFAIL</t>
+  </si>
+  <si>
+    <t>OLS7910F</t>
+  </si>
+  <si>
+    <t>ols_wt_excode: Exit Code must be between 0 and 255.</t>
+  </si>
+  <si>
+    <t>OLS7030F</t>
+  </si>
+  <si>
+    <t>EX_CODE</t>
+  </si>
+  <si>
+    <t>function</t>
+  </si>
+  <si>
+    <t>Program starts</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #1, &lt;arg_1&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #2, &lt;arg_2&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #3, &lt;arg_3&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #4, &lt;arg_4&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #5, &lt;arg_5&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #6, &lt;arg_6&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #7, &lt;arg_7&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #8, &lt;arg_8&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #9, &lt;arg_9&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #10, &lt;arg_10&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #11, &lt;arg_11&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #12, &lt;arg_12&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #13, &lt;arg_13&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #14, &lt;arg_14&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #15, &lt;arg_15&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #16, &lt;arg_16&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #17, &lt;arg_17&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #18, &lt;arg_18&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #19, &lt;arg_19&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ols_function&gt;: Missing Argument #20, &lt;arg_20&gt;</t>
+  </si>
+  <si>
+    <t>assert: Assertion Fail. &lt;condition&gt;, &lt;filename&gt;, line &lt;line_number&gt;</t>
+  </si>
+  <si>
+    <t>OLS7050</t>
+  </si>
+  <si>
+    <t>ols_tap_print_test_plan</t>
+  </si>
+  <si>
+    <t>ols_tap_print_test_plan: Argument no_test must be greater then 0</t>
+  </si>
+  <si>
+    <t>OLS7051</t>
+  </si>
+  <si>
+    <t>ols_tap_print_test_plan: Argument no_test must be a natural number</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +272,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -115,9 +305,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,78 +589,462 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="55.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" t="s">
+        <v>37</v>
+      </c>
+      <c r="D36" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Save error messages and man source.
</commit_message>
<xml_diff>
--- a/var/ols_error_messages.xlsx
+++ b/var/ols_error_messages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\b-lib-olaus-J70091652\var\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92495FAC-B480-4B03-8979-6E4142971A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82260F1F-5594-4009-AD69-B1832A6BF69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="3765" windowWidth="45030" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="86">
   <si>
     <t>Error Number</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Error Message</t>
   </si>
   <si>
-    <t>FUNCNAME</t>
-  </si>
-  <si>
     <t>OLS7001F</t>
   </si>
   <si>
@@ -56,9 +53,6 @@
     <t>OLS7002F</t>
   </si>
   <si>
-    <t>Exit Code must be between 0 and 255.</t>
-  </si>
-  <si>
     <t>OLS1000F</t>
   </si>
   <si>
@@ -80,9 +74,6 @@
     <t>OLS7005F</t>
   </si>
   <si>
-    <t>Missing Argument #1.</t>
-  </si>
-  <si>
     <t>Argument #1 is less than or equal 0.</t>
   </si>
   <si>
@@ -255,23 +246,64 @@
   </si>
   <si>
     <t>ols_tap_print_test_plan: Argument no_test must be a natural number</t>
+  </si>
+  <si>
+    <t>OLS7070</t>
+  </si>
+  <si>
+    <t>is_csv</t>
+  </si>
+  <si>
+    <t>EX_NOINPUT</t>
+  </si>
+  <si>
+    <t>is_csv: &lt;csv_file_name&gt; does not exist or is not a normal file</t>
+  </si>
+  <si>
+    <t>OLS7071</t>
+  </si>
+  <si>
+    <t>EX_INFO</t>
+  </si>
+  <si>
+    <t>is_csv: &lt;csv_file_name&gt; does not have a "csv" extention</t>
+  </si>
+  <si>
+    <t>OLS7072</t>
+  </si>
+  <si>
+    <t>build_append</t>
+  </si>
+  <si>
+    <t>build-append: '$FILENAME' is not readable</t>
+  </si>
+  <si>
+    <t>OLS7073</t>
+  </si>
+  <si>
+    <t>EX_MISSINGFILE</t>
+  </si>
+  <si>
+    <t>build-append: '$LIB_NAME' is does not exist</t>
+  </si>
+  <si>
+    <t>OLS7074</t>
+  </si>
+  <si>
+    <t>EX_CANTCREAT</t>
+  </si>
+  <si>
+    <t>build-append: '$LIB_NAME' is not writeable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -305,10 +337,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -589,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -598,78 +629,55 @@
     <col min="5" max="5" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -677,21 +685,52 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
         <v>46</v>
@@ -699,13 +738,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
         <v>47</v>
@@ -713,13 +752,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
         <v>48</v>
@@ -727,13 +766,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
         <v>49</v>
@@ -741,13 +780,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
         <v>50</v>
@@ -755,13 +794,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
         <v>51</v>
@@ -772,10 +811,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
         <v>52</v>
@@ -786,10 +825,10 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
         <v>53</v>
@@ -800,10 +839,10 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
         <v>54</v>
@@ -814,10 +853,10 @@
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
         <v>55</v>
@@ -828,10 +867,10 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
         <v>56</v>
@@ -842,10 +881,10 @@
         <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D21" t="s">
         <v>57</v>
@@ -856,10 +895,10 @@
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D22" t="s">
         <v>58</v>
@@ -870,10 +909,10 @@
         <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D23" t="s">
         <v>59</v>
@@ -884,10 +923,10 @@
         <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D24" t="s">
         <v>60</v>
@@ -898,10 +937,10 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D25" t="s">
         <v>61</v>
@@ -912,10 +951,10 @@
         <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D26" t="s">
         <v>62</v>
@@ -926,10 +965,10 @@
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D27" t="s">
         <v>63</v>
@@ -940,111 +979,139 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D28" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" t="s">
-        <v>65</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B30" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C30" t="s">
         <v>37</v>
       </c>
       <c r="D30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D31" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="C33" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D33" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>43</v>
-      </c>
-      <c r="B34" t="s">
-        <v>4</v>
-      </c>
-      <c r="C34" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" t="s">
         <v>71</v>
       </c>
-      <c r="B35" t="s">
-        <v>69</v>
-      </c>
       <c r="C35" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="D35" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="D36" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" t="s">
         <v>72</v>
+      </c>
+      <c r="D37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" t="s">
+        <v>81</v>
+      </c>
+      <c r="D38" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>83</v>
+      </c>
+      <c r="B39" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" t="s">
+        <v>84</v>
+      </c>
+      <c r="D39" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update error messages for build-append
</commit_message>
<xml_diff>
--- a/var/ols_error_messages.xlsx
+++ b/var/ols_error_messages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\b-lib-olaus-J70091652\var\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82260F1F-5594-4009-AD69-B1832A6BF69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9157250B-C918-403E-BC74-3655DE9CB77C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="3765" windowWidth="45030" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="88">
   <si>
     <t>Error Number</t>
   </si>
@@ -233,24 +233,15 @@
     <t>assert: Assertion Fail. &lt;condition&gt;, &lt;filename&gt;, line &lt;line_number&gt;</t>
   </si>
   <si>
-    <t>OLS7050</t>
-  </si>
-  <si>
     <t>ols_tap_print_test_plan</t>
   </si>
   <si>
     <t>ols_tap_print_test_plan: Argument no_test must be greater then 0</t>
   </si>
   <si>
-    <t>OLS7051</t>
-  </si>
-  <si>
     <t>ols_tap_print_test_plan: Argument no_test must be a natural number</t>
   </si>
   <si>
-    <t>OLS7070</t>
-  </si>
-  <si>
     <t>is_csv</t>
   </si>
   <si>
@@ -260,40 +251,55 @@
     <t>is_csv: &lt;csv_file_name&gt; does not exist or is not a normal file</t>
   </si>
   <si>
-    <t>OLS7071</t>
-  </si>
-  <si>
     <t>EX_INFO</t>
   </si>
   <si>
     <t>is_csv: &lt;csv_file_name&gt; does not have a "csv" extention</t>
   </si>
   <si>
-    <t>OLS7072</t>
-  </si>
-  <si>
     <t>build_append</t>
   </si>
   <si>
     <t>build-append: '$FILENAME' is not readable</t>
   </si>
   <si>
-    <t>OLS7073</t>
-  </si>
-  <si>
     <t>EX_MISSINGFILE</t>
   </si>
   <si>
-    <t>build-append: '$LIB_NAME' is does not exist</t>
-  </si>
-  <si>
-    <t>OLS7074</t>
-  </si>
-  <si>
     <t>EX_CANTCREAT</t>
   </si>
   <si>
     <t>build-append: '$LIB_NAME' is not writeable</t>
+  </si>
+  <si>
+    <t>OLS7051F</t>
+  </si>
+  <si>
+    <t>OLS7050F</t>
+  </si>
+  <si>
+    <t>OLS7070F</t>
+  </si>
+  <si>
+    <t>OLS7071I</t>
+  </si>
+  <si>
+    <t>OLS7072F</t>
+  </si>
+  <si>
+    <t>OLS7073F</t>
+  </si>
+  <si>
+    <t>OLS7074F</t>
+  </si>
+  <si>
+    <t>OLS7075F</t>
+  </si>
+  <si>
+    <t>build-append: '$LIB_NAME' does not exist</t>
+  </si>
+  <si>
+    <t>build-append: '$FILENAME' is not does not exist</t>
   </si>
 </sst>
 </file>
@@ -620,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -1018,100 +1024,114 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="B32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" t="s">
         <v>66</v>
-      </c>
-      <c r="C32" t="s">
-        <v>34</v>
-      </c>
-      <c r="D32" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="B33" t="s">
-        <v>66</v>
-      </c>
       <c r="C33" t="s">
         <v>34</v>
       </c>
       <c r="D33" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" t="s">
         <v>70</v>
-      </c>
-      <c r="B35" t="s">
-        <v>71</v>
-      </c>
-      <c r="C35" t="s">
-        <v>72</v>
-      </c>
-      <c r="D35" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" t="s">
         <v>71</v>
       </c>
-      <c r="C36" t="s">
-        <v>75</v>
-      </c>
       <c r="D36" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B37" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C38" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D38" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B39" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C39" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="D39" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>85</v>
+      </c>
+      <c r="B40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
+        <v>76</v>
+      </c>
+      <c r="D40" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>